<commit_message>
Upload to JLCPCB - Rel B
</commit_message>
<xml_diff>
--- a/PCB Assembly/USB-SW-B/BOM Basic.xlsx
+++ b/PCB Assembly/USB-SW-B/BOM Basic.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="88">
   <si>
     <t>Line #</t>
   </si>
@@ -45,6 +45,15 @@
     <t>Mount</t>
   </si>
   <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>Conn Post Header - PWM Fan - 90 Deg - 4 Pos - Series KK254</t>
+  </si>
+  <si>
+    <t>Through Hole</t>
+  </si>
+  <si>
     <t>Q1</t>
   </si>
   <si>
@@ -133,24 +142,6 @@
   </si>
   <si>
     <t>JST</t>
-  </si>
-  <si>
-    <t>Through Hole</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>J2</t>
-  </si>
-  <si>
-    <t>CO975</t>
-  </si>
-  <si>
-    <t>Conn Post Header - PWM Fan - 90 Deg - 4 Pos - Series KK254</t>
-  </si>
-  <si>
-    <t>Moddy</t>
   </si>
   <si>
     <t>7</t>
@@ -546,10 +537,12 @@
     <xf xxid="44" numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyBorder="1" quotePrefix="1"/>
     <xf xxid="45" numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyBorder="1"/>
     <xf xxid="46" numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyBorder="1"/>
-    <xf xxid="47" numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyBorder="1" quotePrefix="1"/>
-    <xf xxid="48" numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyBorder="1" quotePrefix="1"/>
-    <xf xxid="49" numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyBorder="1" applyFill="1"/>
-    <xf xxid="50" numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyBorder="1" applyFill="1"/>
+    <xf xxid="47" numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyBorder="1"/>
+    <xf xxid="48" numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyBorder="1"/>
+    <xf xxid="49" numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="50" numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyBorder="1" quotePrefix="1"/>
+    <xf xxid="51" numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyBorder="1" applyFill="1"/>
+    <xf xxid="52" numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyBorder="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -577,28 +570,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="30" t="s">
+      <c r="C1" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="30" t="s">
+      <c r="E1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="30" t="s">
+      <c r="F1" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="30" t="s">
+      <c r="G1" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="30" t="s">
+      <c r="H1" s="32" t="s">
         <v>8</v>
       </c>
     </row>
@@ -607,439 +600,431 @@
       <c r="B2" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="19"/>
+      <c r="D2" s="19">
+        <v>1</v>
+      </c>
+      <c r="E2" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="19">
-        <v>1</v>
-      </c>
-      <c r="E2" s="21" t="s">
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="21" t="s">
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="28"/>
+      <c r="B3" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="C3" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="21" t="s">
+      <c r="D3" s="15">
+        <v>1</v>
+      </c>
+      <c r="E3" s="17" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="28" t="s">
+      <c r="F3" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="15">
-        <v>1</v>
-      </c>
-      <c r="E3" s="17" t="s">
+      <c r="G3" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="B4" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="28" t="s">
+      <c r="C4" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="D4" s="15">
+        <v>1</v>
+      </c>
+      <c r="E4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="F4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="15">
+      <c r="G4" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="15">
         <v>3</v>
       </c>
-      <c r="E4" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="17" t="s">
+      <c r="E5" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="15">
+      <c r="F5" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="15">
         <v>2</v>
       </c>
-      <c r="E5" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="28" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="17" t="s">
+      <c r="E6" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="F6" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="15">
-        <v>1</v>
-      </c>
-      <c r="E6" s="17" t="s">
+      <c r="G6" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="B7" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="28" t="s">
+      <c r="C7" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="D7" s="15">
+        <v>1</v>
+      </c>
+      <c r="E7" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="F7" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="15">
-        <v>1</v>
-      </c>
-      <c r="E7" s="17" t="s">
+      <c r="G7" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="B8" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H7" s="17" t="s">
+      <c r="C8" s="17" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="28" t="s">
+      <c r="D8" s="15">
+        <v>1</v>
+      </c>
+      <c r="E8" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="F8" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="G8" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="15">
-        <v>1</v>
-      </c>
-      <c r="E8" s="17" t="s">
+      <c r="B9" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="C9" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="28" t="s">
+      <c r="D9" s="15">
+        <v>1</v>
+      </c>
+      <c r="E9" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="F9" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="G9" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="D9" s="15">
-        <v>1</v>
-      </c>
-      <c r="E9" s="17" t="s">
+      <c r="B10" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="C10" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="28" t="s">
+      <c r="D10" s="15">
+        <v>1</v>
+      </c>
+      <c r="E10" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="F10" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="G10" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="15">
-        <v>1</v>
-      </c>
-      <c r="E10" s="17" t="s">
+      <c r="B11" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="C11" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="G10" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="28" t="s">
+      <c r="D11" s="15">
+        <v>1</v>
+      </c>
+      <c r="E11" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="F11" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="G11" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="15">
-        <v>1</v>
-      </c>
-      <c r="E11" s="17" t="s">
+      <c r="B12" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="C12" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="G11" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="28" t="s">
+      <c r="D12" s="15">
+        <v>1</v>
+      </c>
+      <c r="E12" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="F12" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="B13" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="D12" s="15">
-        <v>1</v>
-      </c>
-      <c r="E12" s="17" t="s">
+      <c r="C13" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="F12" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H12" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="28" t="s">
+      <c r="D13" s="15">
+        <v>1</v>
+      </c>
+      <c r="E13" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="F13" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="G13" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="30" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="15">
-        <v>1</v>
-      </c>
-      <c r="E13" s="17" t="s">
+      <c r="B14" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="C14" s="17" t="s">
         <v>68</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="C14" s="17" t="s">
-        <v>71</v>
       </c>
       <c r="D14" s="15">
         <v>3</v>
       </c>
       <c r="E14" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="G14" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="C15" s="17" t="s">
         <v>73</v>
-      </c>
-      <c r="G14" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" s="17" t="s">
-        <v>76</v>
       </c>
       <c r="D15" s="15">
         <v>3</v>
       </c>
       <c r="E15" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="30" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C16" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="F15" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="G15" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="28" t="s">
+      <c r="D16" s="15">
+        <v>1</v>
+      </c>
+      <c r="E16" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="F16" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="G16" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16" s="17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="D16" s="15">
-        <v>1</v>
-      </c>
-      <c r="E16" s="17" t="s">
+      <c r="B17" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="C17" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="G16" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="28" t="s">
+      <c r="D17" s="15">
+        <v>1</v>
+      </c>
+      <c r="E17" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="F17" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="G17" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="B18" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="15">
-        <v>1</v>
-      </c>
-      <c r="E17" s="17" t="s">
+      <c r="C18" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="F17" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="G17" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="17" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" s="28" t="s">
+      <c r="D18" s="15">
+        <v>1</v>
+      </c>
+      <c r="E18" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="B18" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>89</v>
-      </c>
-      <c r="D18" s="15">
-        <v>1</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>90</v>
-      </c>
       <c r="F18" s="17" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>